<commit_message>
Address PR review: validate initial values, fix docs, reuse helper
Resolve reviewer feedback on PR #973:
- readInitialValuesFromXLS(): hard-error on missing/non-numeric Value
  (new errorMissingValuesInInitialValues) and on non-logical "Is Present"
  cells (new errorInvalidIsPresentInInitialValues) instead of silently
  coercing to NA; validate before mutating the accumulators
- readScenarioConfigurationFromExcel(): reuse .splitCommaString() for the
  InitialValuesSet column instead of a duplicated inline scan()
- .validateParametersStructure(): enforce equal lengths of paths/values/
  units, matching the long-standing error message
- vignette: correct the three places that wrongly claimed empty Units
  defaults to base units (units/values are mandatory for present molecules)

Tests: new fixture sheets (MissingValue, BadIsPresent) and tests for the
value, Is Present, and validator length checks.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/data/InitialValues.xlsx
+++ b/tests/data/InitialValues.xlsx
@@ -10,8 +10,10 @@
     <sheet name="ValidSheet" sheetId="1" r:id="rId1"/>
     <sheet name="SecondSheet" sheetId="2" r:id="rId2"/>
     <sheet name="MissingUnits" sheetId="3" r:id="rId3"/>
-    <sheet name="AllAbsent" sheetId="4" r:id="rId4"/>
-    <sheet name="InvalidSheet" sheetId="5" r:id="rId5"/>
+    <sheet name="MissingValue" sheetId="4" r:id="rId4"/>
+    <sheet name="BadIsPresent" sheetId="5" r:id="rId5"/>
+    <sheet name="AllAbsent" sheetId="6" r:id="rId6"/>
+    <sheet name="InvalidSheet" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -633,7 +635,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -685,10 +687,7 @@
         </is>
       </c>
       <c r="C2" t="b">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -699,35 +698,6 @@
         <v>1</v>
       </c>
       <c r="G2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Organism|Kidney</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>µmol</t>
-        </is>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3" t="b">
         <v>0</v>
       </c>
     </row>
@@ -738,6 +708,189 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Container Path</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Molecule Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Is Present</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Scale Divisor</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Neg. Values Allowed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Organism|Liver</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D2">
+        <v>0.5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>µmol</t>
+        </is>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Container Path</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Molecule Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Is Present</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Scale Divisor</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Neg. Values Allowed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Organism|Liver</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C2" t="b">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0.5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>µmol</t>
+        </is>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Organism|Kidney</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C3" t="b">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>µmol</t>
+        </is>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>